<commit_message>
complete db's for plausibility assessment
</commit_message>
<xml_diff>
--- a/input_data/envelope_assignement.xlsx
+++ b/input_data/envelope_assignement.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dominicbuettiker/Documents/GitHub/Parametric-LCA-Urban-Densification/input_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29087214-50B0-F341-BED6-AC3B0ED53E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA6244D9-5D66-134C-A9D7-392BAB2F43F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2620" yWindow="760" windowWidth="27440" windowHeight="16240" xr2:uid="{6CB9E5F3-7970-1640-84D6-E8497AD75D04}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="39">
   <si>
     <t>core</t>
   </si>
@@ -147,13 +147,19 @@
   </si>
   <si>
     <t>roof_ext_finishing_to_attic_cold_replacement</t>
+  </si>
+  <si>
+    <t>eps</t>
+  </si>
+  <si>
+    <t>for modelvalidation with Galamshina et. al 2024</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -163,6 +169,12 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -204,11 +216,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -673,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA30F6C1-CD0F-3A48-B94B-9339DA54F9BC}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.33203125" customWidth="1"/>
@@ -934,6 +948,61 @@
         <v>30</v>
       </c>
     </row>
+    <row r="19" spans="1:6" s="5" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:6" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>